<commit_message>
fix(excel-template): fix dependent department dropdown and restore official institutional branding
</commit_message>
<xml_diff>
--- a/backend/public/templates/jmcfi_user_accounts_template.xlsx
+++ b/backend/public/templates/jmcfi_user_accounts_template.xlsx
@@ -30,10 +30,10 @@
     <t>FOUNDATION, INC.</t>
   </si>
   <si>
-    <t>KJC Compound, Phil-Jap Friendship Highway, Sasa, Davao City, Philippines</t>
-  </si>
-  <si>
-    <t>Portal: www.jmc.edu.ph | communications@jmc.edu.ph | (+639) 994970107</t>
+    <t>KJC Compound, Phil-Jap Friendship Highway, Sasa, Davao City, Phillipines</t>
+  </si>
+  <si>
+    <t>www.jmc.edu.ph    |    communications@jmc.edu.ph</t>
   </si>
   <si>
     <t>Assured • Consistent • Quality Education</t>
@@ -80,40 +80,38 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <color rgb="FF1E3A8A"/>
-      <name val="Georgia"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Old English Text MT"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF374151"/>
-      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <u/>
-      <sz val="8.5"/>
-      <color rgb="FF4B5563"/>
+      <sz val="9"/>
+      <color rgb="FF222222"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8.5"/>
-      <color rgb="FF4B5563"/>
+      <color rgb="FF333333"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <i/>
-      <sz val="8.5"/>
-      <color rgb="FF5B0FB8"/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -173,16 +171,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFE5E7EB"/>
       </left>
       <right style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFE5E7EB"/>
       </right>
       <top style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFE5E7EB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFE5E7EB"/>
       </bottom>
       <diagonal/>
     </border>
@@ -233,13 +231,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>152400</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>981456</xdr:colOff>
+      <xdr:colOff>1030224</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>19431</xdr:rowOff>
+      <xdr:rowOff>68199</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -256,8 +254,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="152400" y="38100"/>
-          <a:ext cx="829056" cy="829056"/>
+          <a:off x="152400" y="57150"/>
+          <a:ext cx="877824" cy="877824"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -558,13 +556,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="18.7109375" customWidth="1"/>
-    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
     <col min="5" max="5" width="20.7109375" customWidth="1"/>
     <col min="6" max="6" width="38.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="24" customHeight="1">
+    <row r="1" spans="1:6" ht="26" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -604,7 +602,7 @@
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="14" customHeight="1">
+    <row r="5" spans="1:6">
       <c r="A5" s="1"/>
       <c r="B5" s="6" t="s">
         <v>4</v>
@@ -614,7 +612,7 @@
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
     </row>
-    <row r="6" spans="1:6" ht="6" customHeight="1">
+    <row r="6" spans="1:6" ht="5" customHeight="1">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -1076,324 +1074,12 @@
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A6:F6"/>
   </mergeCells>
-  <dataValidations count="106">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E8">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E8:E60">
       <formula1>SystemRoles</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F8">
-      <formula1>INDIRECT(SUBSTITUTE($E8, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E9">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F9">
-      <formula1>INDIRECT(SUBSTITUTE($E9, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E10">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F10">
-      <formula1>INDIRECT(SUBSTITUTE($E10, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E11">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F11">
-      <formula1>INDIRECT(SUBSTITUTE($E11, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E12">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F12">
-      <formula1>INDIRECT(SUBSTITUTE($E12, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E13">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F13">
-      <formula1>INDIRECT(SUBSTITUTE($E13, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E14">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F14">
-      <formula1>INDIRECT(SUBSTITUTE($E14, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E15">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F15">
-      <formula1>INDIRECT(SUBSTITUTE($E15, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E16">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F16">
-      <formula1>INDIRECT(SUBSTITUTE($E16, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E17">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F17">
-      <formula1>INDIRECT(SUBSTITUTE($E17, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E18">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F18">
-      <formula1>INDIRECT(SUBSTITUTE($E18, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E19">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F19">
-      <formula1>INDIRECT(SUBSTITUTE($E19, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E20">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F20">
-      <formula1>INDIRECT(SUBSTITUTE($E20, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E21">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F21">
-      <formula1>INDIRECT(SUBSTITUTE($E21, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E22">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F22">
-      <formula1>INDIRECT(SUBSTITUTE($E22, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E23">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F23">
-      <formula1>INDIRECT(SUBSTITUTE($E23, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E24">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F24">
-      <formula1>INDIRECT(SUBSTITUTE($E24, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E25">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F25">
-      <formula1>INDIRECT(SUBSTITUTE($E25, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E26">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F26">
-      <formula1>INDIRECT(SUBSTITUTE($E26, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E27">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F27">
-      <formula1>INDIRECT(SUBSTITUTE($E27, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E28">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F28">
-      <formula1>INDIRECT(SUBSTITUTE($E28, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E29">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F29">
-      <formula1>INDIRECT(SUBSTITUTE($E29, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E30">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F30">
-      <formula1>INDIRECT(SUBSTITUTE($E30, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E31">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F31">
-      <formula1>INDIRECT(SUBSTITUTE($E31, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E32">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F32">
-      <formula1>INDIRECT(SUBSTITUTE($E32, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E33">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F33">
-      <formula1>INDIRECT(SUBSTITUTE($E33, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E34">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F34">
-      <formula1>INDIRECT(SUBSTITUTE($E34, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E35">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F35">
-      <formula1>INDIRECT(SUBSTITUTE($E35, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E36">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F36">
-      <formula1>INDIRECT(SUBSTITUTE($E36, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E37">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F37">
-      <formula1>INDIRECT(SUBSTITUTE($E37, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E38">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F38">
-      <formula1>INDIRECT(SUBSTITUTE($E38, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E39">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F39">
-      <formula1>INDIRECT(SUBSTITUTE($E39, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E40">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F40">
-      <formula1>INDIRECT(SUBSTITUTE($E40, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E41">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F41">
-      <formula1>INDIRECT(SUBSTITUTE($E41, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E42">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F42">
-      <formula1>INDIRECT(SUBSTITUTE($E42, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E43">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F43">
-      <formula1>INDIRECT(SUBSTITUTE($E43, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E44">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F44">
-      <formula1>INDIRECT(SUBSTITUTE($E44, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E45">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F45">
-      <formula1>INDIRECT(SUBSTITUTE($E45, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E46">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F46">
-      <formula1>INDIRECT(SUBSTITUTE($E46, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E47">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F47">
-      <formula1>INDIRECT(SUBSTITUTE($E47, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E48">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F48">
-      <formula1>INDIRECT(SUBSTITUTE($E48, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E49">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F49">
-      <formula1>INDIRECT(SUBSTITUTE($E49, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E50">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F50">
-      <formula1>INDIRECT(SUBSTITUTE($E50, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E51">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F51">
-      <formula1>INDIRECT(SUBSTITUTE($E51, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E52">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F52">
-      <formula1>INDIRECT(SUBSTITUTE($E52, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E53">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F53">
-      <formula1>INDIRECT(SUBSTITUTE($E53, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E54">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F54">
-      <formula1>INDIRECT(SUBSTITUTE($E54, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E55">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F55">
-      <formula1>INDIRECT(SUBSTITUTE($E55, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E56">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F56">
-      <formula1>INDIRECT(SUBSTITUTE($E56, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E57">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F57">
-      <formula1>INDIRECT(SUBSTITUTE($E57, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E58">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F58">
-      <formula1>INDIRECT(SUBSTITUTE($E58, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E59">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F59">
-      <formula1>INDIRECT(SUBSTITUTE($E59, " ", "_"))</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Approver, Requestor, Admin)" sqref="E60">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a department that belongs to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F60">
-      <formula1>INDIRECT(SUBSTITUTE($E60, " ", "_"))</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F8:F60">
+      <formula1>INDIRECT($E8)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
chore: sync regenerated template files from dry run verification
</commit_message>
<xml_diff>
--- a/backend/public/templates/jmcfi_user_accounts_template.xlsx
+++ b/backend/public/templates/jmcfi_user_accounts_template.xlsx
@@ -11,10 +11,10 @@
     <sheet name="SystemData" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="Admin">SystemData!$Z$1</definedName>
-    <definedName name="Approver">SystemData!$Z$1</definedName>
+    <definedName name="Admin">SystemData!$D$1:$D$1</definedName>
+    <definedName name="Approver">SystemData!$C$1:$C$5</definedName>
     <definedName name="Empty_List">SystemData!$Z$1</definedName>
-    <definedName name="Requestor">SystemData!$Z$1</definedName>
+    <definedName name="Requestor">SystemData!$B$1:$B$3</definedName>
     <definedName name="SystemRoles">SystemData!$A$1:$A$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>JOSE MARIA COLLEGE</t>
   </si>
@@ -64,6 +64,24 @@
   </si>
   <si>
     <t>Admin</t>
+  </si>
+  <si>
+    <t>BSA</t>
+  </si>
+  <si>
+    <t>College of Information Technology</t>
+  </si>
+  <si>
+    <t>Psyc</t>
+  </si>
+  <si>
+    <t>Institutional Marketing Communication</t>
+  </si>
+  <si>
+    <t>Vice President of Academic Affairs</t>
+  </si>
+  <si>
+    <t>Information Technology Office</t>
   </si>
 </sst>
 </file>
@@ -1089,22 +1107,53 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:1">
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:1">
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="C5" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(excel-import): ensure imported users can authenticate and log in securely
- Hash passwords using Hash::make() matching standard account creation
- Normalize email addresses to lowercase to prevent PostgreSQL case-sensitivity login mismatch
- Add email_verified_at to User fillable attributes so imported accounts are pre-verified
- Handle account upsert if user already exists instead of silently skipping
- Sync user roles using Spatie syncRoles and assign matching departments
- Robustly parse sparse rows in Excel import preventing template header search failure
- Return HTTP 422 with structured errors when accounts fail to import
- Add backend automated tests covering bulk import, authentication, and validation
</commit_message>
<xml_diff>
--- a/backend/public/templates/jmcfi_user_accounts_template.xlsx
+++ b/backend/public/templates/jmcfi_user_accounts_template.xlsx
@@ -11,10 +11,10 @@
     <sheet name="SystemData" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="Admin">SystemData!$D$1:$D$1</definedName>
-    <definedName name="Approver">SystemData!$C$1:$C$5</definedName>
+    <definedName name="Admin">SystemData!$Z$1</definedName>
+    <definedName name="Approver">SystemData!$Z$1</definedName>
     <definedName name="Empty_List">SystemData!$Z$1</definedName>
-    <definedName name="Requestor">SystemData!$B$1:$B$3</definedName>
+    <definedName name="Requestor">SystemData!$Z$1</definedName>
     <definedName name="SystemRoles">SystemData!$A$1:$A$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>JOSE MARIA COLLEGE</t>
   </si>
@@ -64,24 +64,6 @@
   </si>
   <si>
     <t>Admin</t>
-  </si>
-  <si>
-    <t>BSA</t>
-  </si>
-  <si>
-    <t>College of Information Technology</t>
-  </si>
-  <si>
-    <t>Psyc</t>
-  </si>
-  <si>
-    <t>Institutional Marketing Communication</t>
-  </si>
-  <si>
-    <t>Vice President of Academic Affairs</t>
-  </si>
-  <si>
-    <t>Information Technology Office</t>
   </si>
 </sst>
 </file>
@@ -1107,53 +1089,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+    </row>
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+    </row>
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="C5" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(excel-template): fix role-based dependent department dropdown and restore institutional header branding
</commit_message>
<xml_diff>
--- a/backend/public/templates/jmcfi_user_accounts_template.xlsx
+++ b/backend/public/templates/jmcfi_user_accounts_template.xlsx
@@ -30,10 +30,10 @@
     <t>FOUNDATION, INC.</t>
   </si>
   <si>
-    <t>KJC Compound, Phil-Jap Friendship Highway, Sasa, Davao City, Phillipines</t>
+    <t>KJC Compound, Phil-Jap Friendship Highway, Sasa, Davao City, Philippines</t>
   </si>
   <si>
-    <t>www.jmc.edu.ph    |    communications@jmc.edu.ph</t>
+    <t>Portal: www.jmc.edu.ph | communications@jmc.edu.ph | (+639) 994970107</t>
   </si>
   <si>
     <t>Assured • Consistent • Quality Education</t>
@@ -80,38 +80,40 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="Old English Text MT"/>
+      <sz val="16"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Georgia"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <color rgb="FF374151"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <u/>
-      <sz val="9"/>
-      <color rgb="FF222222"/>
+      <sz val="8.5"/>
+      <color rgb="FF4B5563"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8.5"/>
-      <color rgb="FF333333"/>
+      <color rgb="FF4B5563"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <i/>
       <sz val="9"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF5B0FB8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -171,16 +173,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="FFD1D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="FFD1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="FFD1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="FFD1D5DB"/>
       </bottom>
       <diagonal/>
     </border>
@@ -188,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -208,7 +210,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -231,13 +232,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>152400</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1030224</xdr:colOff>
+      <xdr:colOff>981456</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>68199</xdr:rowOff>
+      <xdr:rowOff>19431</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -254,8 +255,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="152400" y="57150"/>
-          <a:ext cx="877824" cy="877824"/>
+          <a:off x="152400" y="38100"/>
+          <a:ext cx="829056" cy="829056"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -562,7 +563,7 @@
     <col min="6" max="6" width="38.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="26" customHeight="1">
+    <row r="1" spans="1:6" ht="24" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -612,474 +613,791 @@
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
     </row>
-    <row r="6" spans="1:6" ht="5" customHeight="1">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-    </row>
-    <row r="7" spans="1:6" ht="26" customHeight="1">
-      <c r="A7" s="8" t="s">
+    <row r="6" spans="1:6" ht="26" customHeight="1">
+      <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>10</v>
       </c>
     </row>
+    <row r="7" spans="1:6" ht="20" customHeight="1">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+    </row>
     <row r="8" spans="1:6" ht="20" customHeight="1">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:6" ht="20" customHeight="1">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:6" ht="20" customHeight="1">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:6" ht="20" customHeight="1">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="20" customHeight="1">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" ht="20" customHeight="1">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" ht="20" customHeight="1">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6" ht="20" customHeight="1">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:6" ht="20" customHeight="1">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:6" ht="20" customHeight="1">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:6" ht="20" customHeight="1">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:6" ht="20" customHeight="1">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:6" ht="20" customHeight="1">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:6" ht="20" customHeight="1">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:6" ht="20" customHeight="1">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:6" ht="20" customHeight="1">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:6" ht="20" customHeight="1">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:6" ht="20" customHeight="1">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
+      <c r="A25" s="8"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:6" ht="20" customHeight="1">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:6" ht="20" customHeight="1">
-      <c r="A27" s="9"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
+      <c r="A27" s="8"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6" ht="20" customHeight="1">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
+      <c r="A28" s="8"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:6" ht="20" customHeight="1">
-      <c r="A29" s="9"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
+      <c r="A29" s="8"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:6" ht="20" customHeight="1">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
+      <c r="A30" s="8"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6" ht="20" customHeight="1">
-      <c r="A31" s="9"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
+      <c r="A31" s="8"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:6" ht="20" customHeight="1">
-      <c r="A32" s="9"/>
-      <c r="B32" s="9"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:6" ht="20" customHeight="1">
-      <c r="A33" s="9"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:6" ht="20" customHeight="1">
-      <c r="A34" s="9"/>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
+      <c r="A34" s="8"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:6" ht="20" customHeight="1">
-      <c r="A35" s="9"/>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
+      <c r="A35" s="8"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:6" ht="20" customHeight="1">
-      <c r="A36" s="9"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
+      <c r="A36" s="8"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
     </row>
     <row r="37" spans="1:6" ht="20" customHeight="1">
-      <c r="A37" s="9"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
+      <c r="A37" s="8"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
     </row>
     <row r="38" spans="1:6" ht="20" customHeight="1">
-      <c r="A38" s="9"/>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
+      <c r="A38" s="8"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:6" ht="20" customHeight="1">
-      <c r="A39" s="9"/>
-      <c r="B39" s="9"/>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
+      <c r="A39" s="8"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:6" ht="20" customHeight="1">
-      <c r="A40" s="9"/>
-      <c r="B40" s="9"/>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
+      <c r="A40" s="8"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
     </row>
     <row r="41" spans="1:6" ht="20" customHeight="1">
-      <c r="A41" s="9"/>
-      <c r="B41" s="9"/>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
+      <c r="A41" s="8"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
     </row>
     <row r="42" spans="1:6" ht="20" customHeight="1">
-      <c r="A42" s="9"/>
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
+      <c r="A42" s="8"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
     </row>
     <row r="43" spans="1:6" ht="20" customHeight="1">
-      <c r="A43" s="9"/>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
+      <c r="A43" s="8"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
     </row>
     <row r="44" spans="1:6" ht="20" customHeight="1">
-      <c r="A44" s="9"/>
-      <c r="B44" s="9"/>
-      <c r="C44" s="9"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
+      <c r="A44" s="8"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
     </row>
     <row r="45" spans="1:6" ht="20" customHeight="1">
-      <c r="A45" s="9"/>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
+      <c r="A45" s="8"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
     </row>
     <row r="46" spans="1:6" ht="20" customHeight="1">
-      <c r="A46" s="9"/>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9"/>
+      <c r="A46" s="8"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8"/>
     </row>
     <row r="47" spans="1:6" ht="20" customHeight="1">
-      <c r="A47" s="9"/>
-      <c r="B47" s="9"/>
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
+      <c r="A47" s="8"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
     </row>
     <row r="48" spans="1:6" ht="20" customHeight="1">
-      <c r="A48" s="9"/>
-      <c r="B48" s="9"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="9"/>
+      <c r="A48" s="8"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
     </row>
     <row r="49" spans="1:6" ht="20" customHeight="1">
-      <c r="A49" s="9"/>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="9"/>
+      <c r="A49" s="8"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
+      <c r="F49" s="8"/>
     </row>
     <row r="50" spans="1:6" ht="20" customHeight="1">
-      <c r="A50" s="9"/>
-      <c r="B50" s="9"/>
-      <c r="C50" s="9"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="9"/>
+      <c r="A50" s="8"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
     </row>
     <row r="51" spans="1:6" ht="20" customHeight="1">
-      <c r="A51" s="9"/>
-      <c r="B51" s="9"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="9"/>
+      <c r="A51" s="8"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="8"/>
     </row>
     <row r="52" spans="1:6" ht="20" customHeight="1">
-      <c r="A52" s="9"/>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="9"/>
+      <c r="A52" s="8"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
     </row>
     <row r="53" spans="1:6" ht="20" customHeight="1">
-      <c r="A53" s="9"/>
-      <c r="B53" s="9"/>
-      <c r="C53" s="9"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="9"/>
+      <c r="A53" s="8"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="8"/>
+      <c r="F53" s="8"/>
     </row>
     <row r="54" spans="1:6" ht="20" customHeight="1">
-      <c r="A54" s="9"/>
-      <c r="B54" s="9"/>
-      <c r="C54" s="9"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
+      <c r="A54" s="8"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
     </row>
     <row r="55" spans="1:6" ht="20" customHeight="1">
-      <c r="A55" s="9"/>
-      <c r="B55" s="9"/>
-      <c r="C55" s="9"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="9"/>
-      <c r="F55" s="9"/>
+      <c r="A55" s="8"/>
+      <c r="B55" s="8"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8"/>
+      <c r="F55" s="8"/>
     </row>
     <row r="56" spans="1:6" ht="20" customHeight="1">
-      <c r="A56" s="9"/>
-      <c r="B56" s="9"/>
-      <c r="C56" s="9"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="9"/>
+      <c r="A56" s="8"/>
+      <c r="B56" s="8"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="8"/>
     </row>
     <row r="57" spans="1:6" ht="20" customHeight="1">
-      <c r="A57" s="9"/>
-      <c r="B57" s="9"/>
-      <c r="C57" s="9"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="9"/>
+      <c r="A57" s="8"/>
+      <c r="B57" s="8"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
     </row>
     <row r="58" spans="1:6" ht="20" customHeight="1">
-      <c r="A58" s="9"/>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="9"/>
+      <c r="A58" s="8"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="8"/>
     </row>
     <row r="59" spans="1:6" ht="20" customHeight="1">
-      <c r="A59" s="9"/>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
+      <c r="A59" s="8"/>
+      <c r="B59" s="8"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="8"/>
     </row>
     <row r="60" spans="1:6" ht="20" customHeight="1">
-      <c r="A60" s="9"/>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
+      <c r="A60" s="8"/>
+      <c r="B60" s="8"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="A1:A5"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A6:F6"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E8:E60">
-      <formula1>SystemRoles</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F8:F60">
-      <formula1>INDIRECT($E8)</formula1>
+  <dataValidations count="108">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E7">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F7">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E7="","Empty_List",$E7)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E8">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F8">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E8="","Empty_List",$E8)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E9">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F9">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E9="","Empty_List",$E9)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E10">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F10">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E10="","Empty_List",$E10)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E11">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F11">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E11="","Empty_List",$E11)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E12">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F12">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E12="","Empty_List",$E12)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E13">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F13">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E13="","Empty_List",$E13)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E14">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F14">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E14="","Empty_List",$E14)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E15">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F15">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E15="","Empty_List",$E15)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E16">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F16">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E16="","Empty_List",$E16)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E17">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F17">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E17="","Empty_List",$E17)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E18">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F18">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E18="","Empty_List",$E18)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E19">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F19">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E19="","Empty_List",$E19)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E20">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F20">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E20="","Empty_List",$E20)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E21">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F21">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E21="","Empty_List",$E21)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E22">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F22">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E22="","Empty_List",$E22)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E23">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F23">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E23="","Empty_List",$E23)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E24">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F24">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E24="","Empty_List",$E24)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E25">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F25">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E25="","Empty_List",$E25)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E26">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F26">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E26="","Empty_List",$E26)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E27">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F27">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E27="","Empty_List",$E27)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E28">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F28">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E28="","Empty_List",$E28)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E29">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F29">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E29="","Empty_List",$E29)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E30">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F30">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E30="","Empty_List",$E30)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E31">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F31">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E31="","Empty_List",$E31)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E32">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F32">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E32="","Empty_List",$E32)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E33">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F33">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E33="","Empty_List",$E33)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E34">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F34">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E34="","Empty_List",$E34)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E35">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F35">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E35="","Empty_List",$E35)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E36">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F36">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E36="","Empty_List",$E36)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E37">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F37">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E37="","Empty_List",$E37)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E38">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F38">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E38="","Empty_List",$E38)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E39">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F39">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E39="","Empty_List",$E39)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E40">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F40">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E40="","Empty_List",$E40)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E41">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F41">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E41="","Empty_List",$E41)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E42">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F42">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E42="","Empty_List",$E42)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E43">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F43">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E43="","Empty_List",$E43)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E44">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F44">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E44="","Empty_List",$E44)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E45">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F45">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E45="","Empty_List",$E45)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E46">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F46">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E46="","Empty_List",$E46)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E47">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F47">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E47="","Empty_List",$E47)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E48">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F48">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E48="","Empty_List",$E48)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E49">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F49">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E49="","Empty_List",$E49)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E50">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F50">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E50="","Empty_List",$E50)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E51">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F51">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E51="","Empty_List",$E51)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E52">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F52">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E52="","Empty_List",$E52)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E53">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F53">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E53="","Empty_List",$E53)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E54">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F54">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E54="","Empty_List",$E54)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E55">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F55">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E55="","Empty_List",$E55)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E56">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F56">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E56="","Empty_List",$E56)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E57">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F57">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E57="","Empty_List",$E57)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E58">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F58">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E58="","Empty_List",$E58)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E59">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F59">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E59="","Empty_List",$E59)," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a valid role from the dropdown list." promptTitle="Select Role" prompt="Choose a valid system role (Requestor, Approver, Admin)" sqref="E60">
+      <formula1>SystemRoles</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Department" error="Please select a valid department assigned to the selected role." promptTitle="Select Department" prompt="Select role in Column E first, then choose from role-assigned departments." sqref="F60">
+      <formula1>INDIRECT(SUBSTITUTE(IF($E60="","Empty_List",$E60)," ","_"))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
perf: optimize Excel template generation to serve cached file instantly
</commit_message>
<xml_diff>
--- a/backend/public/templates/jmcfi_user_accounts_template.xlsx
+++ b/backend/public/templates/jmcfi_user_accounts_template.xlsx
@@ -11,10 +11,10 @@
     <sheet name="SystemData" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="Admin">SystemData!$Z$1</definedName>
-    <definedName name="Approver">SystemData!$Z$1</definedName>
+    <definedName name="Admin">SystemData!$D$1:$D$1</definedName>
+    <definedName name="Approver">SystemData!$C$1:$C$5</definedName>
     <definedName name="Empty_List">SystemData!$Z$1</definedName>
-    <definedName name="Requestor">SystemData!$Z$1</definedName>
+    <definedName name="Requestor">SystemData!$B$1:$B$3</definedName>
     <definedName name="SystemRoles">SystemData!$A$1:$A$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>JOSE MARIA COLLEGE</t>
   </si>
@@ -64,6 +64,24 @@
   </si>
   <si>
     <t>Admin</t>
+  </si>
+  <si>
+    <t>BSA</t>
+  </si>
+  <si>
+    <t>College of Information Technology</t>
+  </si>
+  <si>
+    <t>Psyc</t>
+  </si>
+  <si>
+    <t>Institutional Marketing Communication</t>
+  </si>
+  <si>
+    <t>Vice President of Academic Affairs</t>
+  </si>
+  <si>
+    <t>Information Technology Office</t>
   </si>
 </sst>
 </file>
@@ -1407,22 +1425,53 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:1">
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:1">
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="C5" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(templates): sync excel template binaries and base64 constants
</commit_message>
<xml_diff>
--- a/backend/public/templates/jmcfi_user_accounts_template.xlsx
+++ b/backend/public/templates/jmcfi_user_accounts_template.xlsx
@@ -11,10 +11,10 @@
     <sheet name="SystemData" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="Admin">SystemData!$D$1:$D$1</definedName>
-    <definedName name="Approver">SystemData!$C$1:$C$5</definedName>
+    <definedName name="Admin">SystemData!$Z$1</definedName>
+    <definedName name="Approver">SystemData!$Z$1</definedName>
     <definedName name="Empty_List">SystemData!$Z$1</definedName>
-    <definedName name="Requestor">SystemData!$B$1:$B$3</definedName>
+    <definedName name="Requestor">SystemData!$Z$1</definedName>
     <definedName name="SystemRoles">SystemData!$A$1:$A$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>JOSE MARIA COLLEGE</t>
   </si>
@@ -64,24 +64,6 @@
   </si>
   <si>
     <t>Admin</t>
-  </si>
-  <si>
-    <t>BSA</t>
-  </si>
-  <si>
-    <t>College of Information Technology</t>
-  </si>
-  <si>
-    <t>Psyc</t>
-  </si>
-  <si>
-    <t>Institutional Marketing Communication</t>
-  </si>
-  <si>
-    <t>Vice President of Academic Affairs</t>
-  </si>
-  <si>
-    <t>Information Technology Office</t>
   </si>
 </sst>
 </file>
@@ -1425,53 +1407,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+    </row>
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+    </row>
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="C5" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(departments): add program heads management and sidebar badges for approver and requestor
</commit_message>
<xml_diff>
--- a/backend/public/templates/jmcfi_user_accounts_template.xlsx
+++ b/backend/public/templates/jmcfi_user_accounts_template.xlsx
@@ -11,10 +11,10 @@
     <sheet name="SystemData" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="Admin">SystemData!$Z$1</definedName>
-    <definedName name="Approver">SystemData!$Z$1</definedName>
+    <definedName name="Admin">SystemData!$D$1:$D$1</definedName>
+    <definedName name="Approver">SystemData!$C$1:$C$6</definedName>
     <definedName name="Empty_List">SystemData!$Z$1</definedName>
-    <definedName name="Requestor">SystemData!$Z$1</definedName>
+    <definedName name="Requestor">SystemData!$B$1:$B$4</definedName>
     <definedName name="SystemRoles">SystemData!$A$1:$A$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>JOSE MARIA COLLEGE</t>
   </si>
@@ -64,6 +64,27 @@
   </si>
   <si>
     <t>Admin</t>
+  </si>
+  <si>
+    <t>BSA</t>
+  </si>
+  <si>
+    <t>Cobe</t>
+  </si>
+  <si>
+    <t>College of Information Technology</t>
+  </si>
+  <si>
+    <t>Psyc</t>
+  </si>
+  <si>
+    <t>Institutional Marketing Communication</t>
+  </si>
+  <si>
+    <t>Vice President of Academic Affairs</t>
+  </si>
+  <si>
+    <t>Information Technology Office</t>
   </si>
 </sst>
 </file>
@@ -1407,22 +1428,61 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:1">
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:1">
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="C6" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>